<commit_message>
Incluir entradas finales para 14 y 15
</commit_message>
<xml_diff>
--- a/tarea1-gestor-contrasenas/docs/mcu5/excel/04-bitacora-planilla.xlsx
+++ b/tarea1-gestor-contrasenas/docs/mcu5/excel/04-bitacora-planilla.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="2"/>
@@ -4214,6 +4214,53 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Documentación</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Actualizar Excel MCU de controles y bitácora (#14 y #15) — Se regeneró `docs/mcu5/excel/04-bitacora-planilla.xlsx` desde las 79</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>`python scripts/actualizar_excels_mcu.py` desde</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>`bitacora: 79 entradas`; `controles: 25 filas de evidencia actualizadas`.</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>Cierra #14 y #15 de `00-pendientes-entrega.md`.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>